<commit_message>
Ready For QA Automation
</commit_message>
<xml_diff>
--- a/Trails_SystemSetting_SCB/Cypress/fixtures/Bulktrail.xlsx
+++ b/Trails_SystemSetting_SCB/Cypress/fixtures/Bulktrail.xlsx
@@ -450,10 +450,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>DMI0009590352</v>
+        <v>1667</v>
       </c>
       <c r="B2" t="str">
-        <v>1668</v>
+        <v>10145</v>
       </c>
       <c r="C2" t="str">
         <v>no</v>
@@ -465,7 +465,7 @@
         <v>PTP</v>
       </c>
       <c r="F2" t="str">
-        <v>2027/12/22</v>
+        <v>2027-12-22</v>
       </c>
       <c r="G2" t="str">
         <v>109</v>
@@ -477,16 +477,16 @@
         <v>Bulk upload</v>
       </c>
       <c r="J2" t="str">
-        <v>6513867142</v>
+        <v>9697086617</v>
       </c>
       <c r="K2" t="str">
-        <v>Wittingfield</v>
+        <v>Marleneland</v>
       </c>
       <c r="L2" t="str">
-        <v>47907 Devonshire Road</v>
+        <v>88448 Johnson Street</v>
       </c>
       <c r="M2" t="str">
-        <v>esujrykt@yopmail.com</v>
+        <v>lnqswxbh@yopmail.com</v>
       </c>
       <c r="N2" t="str">
         <v>permenant</v>

</xml_diff>